<commit_message>
tabtools: refresh demo output files
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_comptab.xlsx
+++ b/tabtools/demo/demo_comptab.xlsx
@@ -199,13 +199,13 @@
     <t>1.05 (0.98, 1.13)</t>
   </si>
   <si>
-    <t>"aHR = adjusted hazard ratio; CI = confidence interval. Models adjusted for age, sex, and comorbidities."</t>
+    <t>aHR = adjusted hazard ratio; CI = confidence interval. Models adjusted for age, sex, and comorbidities.</t>
   </si>
   <si>
     <t>Table S2. Selected Risk Factors (Name-Based Selection)</t>
   </si>
   <si>
-    <t>"Rows selected by label pattern using rownames() option."</t>
+    <t>Rows selected by label pattern using rownames() option.</t>
   </si>
 </sst>
 </file>

</xml_diff>